<commit_message>
feat: simplify product information forms
</commit_message>
<xml_diff>
--- a/public/templates/货品导入模板.xlsx
+++ b/public/templates/货品导入模板.xlsx
@@ -124,10 +124,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -159,10 +159,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F51"/>
+  <dimension ref="A1:E51"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -413,26 +413,23 @@
         <v>单位</v>
       </c>
       <c r="D1" t="str">
-        <v>货品编码</v>
+        <v>排序</v>
       </c>
       <c r="E1" t="str">
-        <v>排序</v>
-      </c>
-      <c r="F1" t="str">
         <v>启用</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F51"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E51"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D10"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -497,48 +494,34 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>货品编码</v>
+        <v>排序</v>
       </c>
       <c r="B7" t="str">
         <v>否</v>
       </c>
       <c r="C7" t="str">
-        <v>建议填写唯一编码；已有编码相同会更新原货品</v>
-      </c>
-      <c r="D7" t="str">
-        <v>OMG-001</v>
+        <v>非负整数，数字越小越靠前；空白按 0 处理</v>
+      </c>
+      <c r="D7">
+        <v>10</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>排序</v>
+        <v>启用</v>
       </c>
       <c r="B8" t="str">
         <v>否</v>
       </c>
       <c r="C8" t="str">
-        <v>非负整数，数字越小越靠前；空白按 0 处理</v>
-      </c>
-      <c r="D8">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>启用</v>
-      </c>
-      <c r="B9" t="str">
-        <v>否</v>
-      </c>
-      <c r="C9" t="str">
         <v>只填写“是”或“否”；空白默认启用</v>
       </c>
-      <c r="D9" t="str">
+      <c r="D8" t="str">
         <v>是</v>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" t="str">
+    <row r="10">
+      <c r="A10" t="str">
         <v>请在第一张“货品导入”工作表中填写数据，不要修改第一行列名；每行填写一个货品。</v>
       </c>
     </row>
@@ -549,7 +532,7 @@
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:D10"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>